<commit_message>
[umarciano] Push Massive Import AORN Employee
</commit_message>
<xml_diff>
--- a/script/templates/IMPORT_DIPARTIMENTO_E_UOC.xlsx
+++ b/script/templates/IMPORT_DIPARTIMENTO_E_UOC.xlsx
@@ -2694,7 +2694,7 @@
         <v>10</v>
       </c>
       <c r="F51" s="0">
-        <v>29539</v>
+        <v>38426</v>
       </c>
       <c r="G51" s="0" t="s">
         <v>12</v>
@@ -2720,7 +2720,7 @@
         <v>10</v>
       </c>
       <c r="F52" s="0">
-        <v>29539</v>
+        <v>38426</v>
       </c>
       <c r="G52" s="0" t="s">
         <v>12</v>
@@ -2746,7 +2746,7 @@
         <v>10</v>
       </c>
       <c r="F53" s="0">
-        <v>29539</v>
+        <v>38426</v>
       </c>
       <c r="G53" s="0" t="s">
         <v>12</v>

</xml_diff>